<commit_message>
Update CZ26012500 summaries with corrected invoice numbers
Supplier reissued invoices: N.KO = WELLNIT260812A, Bevelling Machines
Europe = WELLNIT260812B. Only the invoice number changed; values,
quantities and weights are unchanged. Duplicate-invoice warning marked
as resolved.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0197ffRNfpzT1VFhp51JAVtf
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Bevelling_Machines_Europe_CZ26012500.xlsx
+++ b/output/HS_Code_Summary_Bevelling_Machines_Europe_CZ26012500.xlsx
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="113">
   <si>
     <t xml:space="preserve">HS Code Summary – JCD 1/2 – Bevelling Machines Europe s.r.o. – zásilka CZ26012500</t>
   </si>
@@ -82,7 +82,7 @@
     <t xml:space="preserve">Faktura</t>
   </si>
   <si>
-    <t xml:space="preserve">WELLNIT260812 ze dne 12.08.2026 – TOTAL USD 70 424 (EXW Lishui)</t>
+    <t xml:space="preserve">WELLNIT260812B ze dne 12.08.2026 – TOTAL USD 70 424 (EXW Lishui) – opravené číslo faktury (27.10.2026); PL nese č. WELLNIT260812</t>
   </si>
   <si>
     <t xml:space="preserve">Incoterm</t>
@@ -316,22 +316,25 @@
     <t xml:space="preserve">Klasifikace: ukosovací stroje = frézovací princip → 8459 69 90 (ostatní frézovací stroje, ne číslicově řízené) odpovídá. POZOR: stejný typ stroje (UZ30) má N.KO pod 8459 29 00 (vrtací stroje) – nekonzistence, viz soubor N.KO.</t>
   </si>
   <si>
-    <t xml:space="preserve">■ PŘIJATÉ DOKUMENTY (e-mail A. Nedvídková 09.10.2026)</t>
+    <t xml:space="preserve">■ PŘIJATÉ DOKUMENTY (e-maily A. Nedvídková 09.10.2026 a 27.10.2026)</t>
   </si>
   <si>
     <t xml:space="preserve">✓ B/L F202618035 (kopie, NOT NEGOTIABLE) – MARY MAERSK 635W, Ningbo → Bremerhaven, place of delivery Mělník, shipped on board 06.09.2026</t>
   </si>
   <si>
-    <t xml:space="preserve">✓ CIPL Bevelling Machines Europe – Invoice + Packing list WELLNIT260812 ze 12.08.2026 (TOTAL USD 70 424, 21 cases)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">✓ CIPL N.KO – Invoice + Packing list WELLNIT260812 ze 12.08.2026 (TOTAL USD 45 396, 8 cases)</t>
+    <t xml:space="preserve">✓ CIPL Bevelling Machines Europe – Invoice WELLNIT260812B (opravená verze 27.10.2026) + Packing list WELLNIT260812, oba ze 12.08.2026 (TOTAL USD 70 424, 21 cases)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">✓ CIPL N.KO – Invoice WELLNIT260812A (opravená verze 27.10.2026) + Packing list WELLNIT260812, oba ze 12.08.2026 (TOTAL USD 45 396, 8 cases)</t>
   </si>
   <si>
     <t xml:space="preserve">✓ Popisy zboží v CZ, HS kódy, materiál a účel – tabulka klienta v těle e-mailu (popisy převzaty doslovně)</t>
   </si>
   <si>
-    <t xml:space="preserve">⚠️ Obě faktury mají STEJNÉ číslo WELLNIT260812 i datum, ale jiného odběratele a jiný obsah → vyžádat od dodavatele potvrzení / unikátní čísla faktur (riziko dotazu celního úřadu u 2 JCD se stejným číslem faktury).</t>
+    <t xml:space="preserve">✓ VYŘEŠENO 27.10.2026: původně měly obě faktury stejné číslo WELLNIT260812. Dodavatel zaslal opravené faktury: N.KO = WELLNIT260812A, Bevelling Machines Europe = WELLNIT260812B. Ověřeno porovnáním s původními doklady: změnilo se POUZE číslo faktury – zboží, množství, ceny, TOTAL, hmotnosti i datum jsou beze změny. Do JCD uvádět nová čísla A/B.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pozn.: packing listy v opravených dokladech stále nesou číslo WELLNIT260812 (bez A/B) – drobnost, obsah PL odpovídá; případně požádat o sjednocení.</t>
   </si>
   <si>
     <t xml:space="preserve">■ ⭐ PREFERENČNÍ VĚTA / COO</t>
@@ -1471,7 +1474,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A31"/>
+  <dimension ref="A1:A32"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="160"/>
@@ -1512,7 +1515,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="23" t="s">
         <v>88</v>
       </c>
@@ -1527,38 +1530,38 @@
         <v>90</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="22" t="s">
+    <row r="11" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="23" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="24" t="s">
+      <c r="A12" s="23" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="22" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="24" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="24" t="s">
+    <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="22" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="22" t="s">
+      <c r="A15" s="24" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="24" t="s">
+      <c r="A16" s="22" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="23" t="s">
+      <c r="A17" s="24" t="s">
         <v>97</v>
       </c>
     </row>
@@ -1568,68 +1571,73 @@
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="24" t="s">
+      <c r="A19" s="23" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="23" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="24" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="24" t="s">
+    <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="23" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="23" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="24" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="24" t="s">
+    <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="23" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="23" t="s">
+      <c r="A24" s="24" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="24" t="s">
+      <c r="A25" s="23" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="23" t="s">
+      <c r="A26" s="24" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="23" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="23" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="23" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="23" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="23" t="s">
         <v>111</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="23" t="s">
+        <v>112</v>
       </c>
     </row>
   </sheetData>

</xml_diff>